<commit_message>
fix: incomplete dashboard column
</commit_message>
<xml_diff>
--- a/backend/data/audit_dashboard_excel_simulation_revised.xlsx
+++ b/backend/data/audit_dashboard_excel_simulation_revised.xlsx
@@ -18,7 +18,7 @@
     <sheet name="Summary" sheetId="3" r:id="rId3"/>
     <sheet name="Backend_Mapping" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -970,8 +970,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="EvidenceDashboardTable" displayName="EvidenceDashboardTable" ref="A1:H31">
-  <tableColumns count="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="EvidenceDashboardTable" displayName="EvidenceDashboardTable" ref="A1:I31">
+  <tableColumns count="9">
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Document ID"/>
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Document"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Standards"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Clause"/>
@@ -1134,1064 +1135,1220 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H100"/>
+  <dimension ref="A1:I100"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="34" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="43" customWidth="1"/>
-    <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="5" max="5" width="19" customWidth="1"/>
-    <col min="6" max="6" width="23" customWidth="1"/>
-    <col min="7" max="7" width="17" customWidth="1"/>
-    <col min="8" max="8" width="55" customWidth="1"/>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="34" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="43" customWidth="1"/>
+    <col min="5" max="5" width="20" customWidth="1"/>
+    <col min="6" max="6" width="19" customWidth="1"/>
+    <col min="7" max="7" width="23" customWidth="1"/>
+    <col min="8" max="8" width="17" customWidth="1"/>
+    <col min="9" max="9" width="55" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="21.4" customHeight="1">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:9" ht="21.4" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Document ID</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="28">
-      <c r="A2" s="4" t="s">
+    <row r="2" spans="1:9" ht="28">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>DOC-0001</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="C2" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="D2" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="E2" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="F2" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="G2" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="8">
+      <c r="H2" s="8">
         <v>46162</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="I2" s="6" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="28">
-      <c r="A3" s="4" t="s">
+    <row r="3" spans="1:9" ht="28">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>DOC-0002</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="C3" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="D3" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="E3" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="F3" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="G3" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="8">
+      <c r="H3" s="8">
         <v>46174</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="I3" s="6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="28">
-      <c r="A4" s="4" t="s">
+    <row r="4" spans="1:9" ht="28">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>DOC-0003</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="C4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="D4" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="E4" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="F4" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="G4" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="G4" s="8">
+      <c r="H4" s="8">
         <v>46188</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="I4" s="6" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="28">
-      <c r="A5" s="4" t="s">
+    <row r="5" spans="1:9" ht="28">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>DOC-0004</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="C5" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="D5" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="E5" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="F5" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="G5" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="G5" s="8">
+      <c r="H5" s="8">
         <v>46193</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="I5" s="6" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="28">
-      <c r="A6" s="4" t="s">
+    <row r="6" spans="1:9" ht="28">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>DOC-0005</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="C6" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="D6" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="E6" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="F6" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="G6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="8">
+      <c r="H6" s="8">
         <v>46202</v>
       </c>
-      <c r="H6" s="6" t="s">
+      <c r="I6" s="6" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="28">
-      <c r="A7" s="4" t="s">
+    <row r="7" spans="1:9" ht="28">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>DOC-0006</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="C7" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="D7" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="E7" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="F7" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="G7" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="G7" s="8">
+      <c r="H7" s="8">
         <v>46210</v>
       </c>
-      <c r="H7" s="6" t="s">
+      <c r="I7" s="6" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="28">
-      <c r="A8" s="4" t="s">
+    <row r="8" spans="1:9" ht="28">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>DOC-0007</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="C8" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="D8" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="E8" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="F8" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="G8" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="G8" s="8">
+      <c r="H8" s="8">
         <v>46217</v>
       </c>
-      <c r="H8" s="6" t="s">
+      <c r="I8" s="6" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="28">
-      <c r="A9" s="4" t="s">
+    <row r="9" spans="1:9" ht="28">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>DOC-0008</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="C9" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="D9" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="E9" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="F9" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="G9" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="G9" s="8">
+      <c r="H9" s="8">
         <v>46224</v>
       </c>
-      <c r="H9" s="6" t="s">
+      <c r="I9" s="6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="28">
-      <c r="A10" s="4" t="s">
+    <row r="10" spans="1:9" ht="28">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>DOC-0009</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="C10" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="D10" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="E10" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="F10" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="F10" s="6" t="s">
+      <c r="G10" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="G10" s="8">
+      <c r="H10" s="8">
         <v>46230</v>
       </c>
-      <c r="H10" s="6" t="s">
+      <c r="I10" s="6" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="28">
-      <c r="A11" s="4" t="s">
+    <row r="11" spans="1:9" ht="28">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>DOC-0010</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="C11" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="D11" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="E11" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="F11" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F11" s="6" t="s">
+      <c r="G11" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G11" s="8">
+      <c r="H11" s="8">
         <v>46237</v>
       </c>
-      <c r="H11" s="6" t="s">
+      <c r="I11" s="6" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="28">
-      <c r="A12" s="4" t="s">
+    <row r="12" spans="1:9" ht="28">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>DOC-0011</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="C12" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="D12" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="E12" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="F12" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F12" s="6" t="s">
+      <c r="G12" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G12" s="8">
+      <c r="H12" s="8">
         <v>46245</v>
       </c>
-      <c r="H12" s="6" t="s">
+      <c r="I12" s="6" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="28">
-      <c r="A13" s="4" t="s">
+    <row r="13" spans="1:9" ht="28">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>DOC-0012</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="C13" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="D13" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="E13" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="F13" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="F13" s="6" t="s">
+      <c r="G13" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="G13" s="8">
+      <c r="H13" s="8">
         <v>46251</v>
       </c>
-      <c r="H13" s="6" t="s">
+      <c r="I13" s="6" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="28">
-      <c r="A14" s="4" t="s">
+    <row r="14" spans="1:9" ht="28">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>DOC-0013</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="C14" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="D14" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="E14" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="F14" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F14" s="6" t="s">
+      <c r="G14" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G14" s="8">
+      <c r="H14" s="8">
         <v>46259</v>
       </c>
-      <c r="H14" s="6" t="s">
+      <c r="I14" s="6" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="28">
-      <c r="A15" s="4" t="s">
+    <row r="15" spans="1:9" ht="28">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>DOC-0014</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="C15" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="D15" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="E15" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="F15" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F15" s="6" t="s">
+      <c r="G15" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G15" s="8">
+      <c r="H15" s="8">
         <v>46266</v>
       </c>
-      <c r="H15" s="6" t="s">
+      <c r="I15" s="6" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="28">
-      <c r="A16" s="4" t="s">
+    <row r="16" spans="1:9" ht="28">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>DOC-0015</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="C16" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="D16" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="E16" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="F16" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="F16" s="6" t="s">
+      <c r="G16" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="G16" s="8">
+      <c r="H16" s="8">
         <v>46273</v>
       </c>
-      <c r="H16" s="6" t="s">
+      <c r="I16" s="6" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="28">
-      <c r="A17" s="4" t="s">
+    <row r="17" spans="1:9" ht="28">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>DOC-0016</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="C17" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="D17" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="D17" s="6" t="s">
+      <c r="E17" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="E17" s="6" t="s">
+      <c r="F17" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F17" s="6" t="s">
+      <c r="G17" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="G17" s="8">
+      <c r="H17" s="8">
         <v>46281</v>
       </c>
-      <c r="H17" s="6" t="s">
+      <c r="I17" s="6" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="28">
-      <c r="A18" s="4" t="s">
+    <row r="18" spans="1:9" ht="28">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>DOC-0017</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="C18" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="D18" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="D18" s="6" t="s">
+      <c r="E18" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="E18" s="6" t="s">
+      <c r="F18" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="F18" s="6" t="s">
+      <c r="G18" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="G18" s="8">
+      <c r="H18" s="8">
         <v>46288</v>
       </c>
-      <c r="H18" s="6" t="s">
+      <c r="I18" s="6" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="28">
-      <c r="A19" s="4" t="s">
+    <row r="19" spans="1:9" ht="28">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>DOC-0018</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="C19" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="D19" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="D19" s="6" t="s">
+      <c r="E19" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="E19" s="6" t="s">
+      <c r="F19" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F19" s="6" t="s">
+      <c r="G19" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G19" s="8">
+      <c r="H19" s="8">
         <v>46295</v>
       </c>
-      <c r="H19" s="6" t="s">
+      <c r="I19" s="6" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="28">
-      <c r="A20" s="4" t="s">
+    <row r="20" spans="1:9" ht="28">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>DOC-0019</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="C20" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="D20" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="D20" s="6" t="s">
+      <c r="E20" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="E20" s="6" t="s">
+      <c r="F20" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F20" s="6" t="s">
+      <c r="G20" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="G20" s="8">
+      <c r="H20" s="8">
         <v>46302</v>
       </c>
-      <c r="H20" s="6" t="s">
+      <c r="I20" s="6" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="28">
-      <c r="A21" s="4" t="s">
+    <row r="21" spans="1:9" ht="28">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>DOC-0020</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="C21" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="D21" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="D21" s="6" t="s">
+      <c r="E21" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="E21" s="6" t="s">
+      <c r="F21" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F21" s="6" t="s">
+      <c r="G21" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G21" s="8">
+      <c r="H21" s="8">
         <v>46309</v>
       </c>
-      <c r="H21" s="6" t="s">
+      <c r="I21" s="6" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="28">
-      <c r="A22" s="4" t="s">
+    <row r="22" spans="1:9" ht="28">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>DOC-0021</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="C22" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="D22" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="D22" s="6" t="s">
+      <c r="E22" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E22" s="6" t="s">
+      <c r="F22" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="F22" s="6" t="s">
+      <c r="G22" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="G22" s="8">
+      <c r="H22" s="8">
         <v>46316</v>
       </c>
-      <c r="H22" s="6" t="s">
+      <c r="I22" s="6" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="28">
-      <c r="A23" s="4" t="s">
+    <row r="23" spans="1:9" ht="28">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>DOC-0022</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="C23" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="D23" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="D23" s="6" t="s">
+      <c r="E23" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="E23" s="6" t="s">
+      <c r="F23" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F23" s="6" t="s">
+      <c r="G23" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G23" s="8">
+      <c r="H23" s="8">
         <v>46323</v>
       </c>
-      <c r="H23" s="6" t="s">
+      <c r="I23" s="6" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="28">
-      <c r="A24" s="4" t="s">
+    <row r="24" spans="1:9" ht="28">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>DOC-0023</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="C24" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="D24" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="D24" s="6" t="s">
+      <c r="E24" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="E24" s="6" t="s">
+      <c r="F24" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="F24" s="6" t="s">
+      <c r="G24" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="G24" s="8">
+      <c r="H24" s="8">
         <v>46330</v>
       </c>
-      <c r="H24" s="6" t="s">
+      <c r="I24" s="6" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="28">
-      <c r="A25" s="4" t="s">
+    <row r="25" spans="1:9" ht="28">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>DOC-0024</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="C25" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="C25" s="6" t="s">
+      <c r="D25" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="D25" s="6" t="s">
+      <c r="E25" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="E25" s="6" t="s">
+      <c r="F25" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F25" s="6" t="s">
+      <c r="G25" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G25" s="8">
+      <c r="H25" s="8">
         <v>46337</v>
       </c>
-      <c r="H25" s="6" t="s">
+      <c r="I25" s="6" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="28">
-      <c r="A26" s="4" t="s">
+    <row r="26" spans="1:9" ht="28">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>DOC-0025</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="B26" s="6" t="s">
+      <c r="C26" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C26" s="6" t="s">
+      <c r="D26" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="D26" s="6" t="s">
+      <c r="E26" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E26" s="6" t="s">
+      <c r="F26" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F26" s="6" t="s">
+      <c r="G26" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="G26" s="8">
+      <c r="H26" s="8">
         <v>46344</v>
       </c>
-      <c r="H26" s="6" t="s">
+      <c r="I26" s="6" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="28">
-      <c r="A27" s="4" t="s">
+    <row r="27" spans="1:9" ht="28">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>DOC-0026</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="C27" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="D27" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="D27" s="6" t="s">
+      <c r="E27" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="E27" s="6" t="s">
+      <c r="F27" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="F27" s="6" t="s">
+      <c r="G27" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="G27" s="8">
+      <c r="H27" s="8">
         <v>46351</v>
       </c>
-      <c r="H27" s="6" t="s">
+      <c r="I27" s="6" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="28">
-      <c r="A28" s="4" t="s">
+    <row r="28" spans="1:9" ht="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>DOC-0027</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="C28" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="C28" s="6" t="s">
+      <c r="D28" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="D28" s="6" t="s">
+      <c r="E28" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="E28" s="6" t="s">
+      <c r="F28" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F28" s="6" t="s">
+      <c r="G28" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G28" s="8">
+      <c r="H28" s="8">
         <v>46358</v>
       </c>
-      <c r="H28" s="6" t="s">
+      <c r="I28" s="6" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="28">
-      <c r="A29" s="4" t="s">
+    <row r="29" spans="1:9" ht="28">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>DOC-0028</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="C29" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="D29" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="D29" s="6" t="s">
+      <c r="E29" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="E29" s="6" t="s">
+      <c r="F29" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="F29" s="6" t="s">
+      <c r="G29" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="G29" s="8">
+      <c r="H29" s="8">
         <v>46365</v>
       </c>
-      <c r="H29" s="6" t="s">
+      <c r="I29" s="6" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="28">
-      <c r="A30" s="4" t="s">
+    <row r="30" spans="1:9" ht="28">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>DOC-0029</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="C30" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="D30" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="D30" s="6" t="s">
+      <c r="E30" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E30" s="6" t="s">
+      <c r="F30" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F30" s="6" t="s">
+      <c r="G30" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G30" s="8">
+      <c r="H30" s="8">
         <v>46372</v>
       </c>
-      <c r="H30" s="6" t="s">
+      <c r="I30" s="6" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="28">
-      <c r="A31" s="5" t="s">
+    <row r="31" spans="1:9" ht="28">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>DOC-0030</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="B31" s="7" t="s">
+      <c r="C31" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C31" s="7" t="s">
+      <c r="D31" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="D31" s="7" t="s">
+      <c r="E31" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E31" s="7" t="s">
+      <c r="F31" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="F31" s="7" t="s">
+      <c r="G31" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="G31" s="9">
+      <c r="H31" s="9">
         <v>46379</v>
       </c>
-      <c r="H31" s="7" t="s">
+      <c r="I31" s="7" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="32" spans="1:8">
-      <c r="G32" s="10"/>
-    </row>
-    <row r="33" spans="7:7">
-      <c r="G33" s="10"/>
-    </row>
-    <row r="34" spans="7:7">
-      <c r="G34" s="10"/>
-    </row>
-    <row r="35" spans="7:7">
-      <c r="G35" s="10"/>
-    </row>
-    <row r="36" spans="7:7">
-      <c r="G36" s="10"/>
-    </row>
-    <row r="37" spans="7:7">
-      <c r="G37" s="10"/>
-    </row>
-    <row r="38" spans="7:7">
-      <c r="G38" s="10"/>
-    </row>
-    <row r="39" spans="7:7">
-      <c r="G39" s="10"/>
-    </row>
-    <row r="40" spans="7:7">
-      <c r="G40" s="10"/>
-    </row>
-    <row r="41" spans="7:7">
-      <c r="G41" s="10"/>
-    </row>
-    <row r="42" spans="7:7">
-      <c r="G42" s="10"/>
-    </row>
-    <row r="43" spans="7:7">
-      <c r="G43" s="10"/>
-    </row>
-    <row r="44" spans="7:7">
-      <c r="G44" s="10"/>
-    </row>
-    <row r="45" spans="7:7">
-      <c r="G45" s="10"/>
-    </row>
-    <row r="46" spans="7:7">
-      <c r="G46" s="10"/>
-    </row>
-    <row r="47" spans="7:7">
-      <c r="G47" s="10"/>
-    </row>
-    <row r="48" spans="7:7">
-      <c r="G48" s="10"/>
-    </row>
-    <row r="49" spans="7:7">
-      <c r="G49" s="10"/>
-    </row>
-    <row r="50" spans="7:7">
-      <c r="G50" s="10"/>
-    </row>
-    <row r="51" spans="7:7">
-      <c r="G51" s="10"/>
-    </row>
-    <row r="52" spans="7:7">
-      <c r="G52" s="10"/>
-    </row>
-    <row r="53" spans="7:7">
-      <c r="G53" s="10"/>
-    </row>
-    <row r="54" spans="7:7">
-      <c r="G54" s="10"/>
-    </row>
-    <row r="55" spans="7:7">
-      <c r="G55" s="10"/>
-    </row>
-    <row r="56" spans="7:7">
-      <c r="G56" s="10"/>
-    </row>
-    <row r="57" spans="7:7">
-      <c r="G57" s="10"/>
-    </row>
-    <row r="58" spans="7:7">
-      <c r="G58" s="10"/>
-    </row>
-    <row r="59" spans="7:7">
-      <c r="G59" s="10"/>
-    </row>
-    <row r="60" spans="7:7">
-      <c r="G60" s="10"/>
-    </row>
-    <row r="61" spans="7:7">
-      <c r="G61" s="10"/>
-    </row>
-    <row r="62" spans="7:7">
-      <c r="G62" s="10"/>
-    </row>
-    <row r="63" spans="7:7">
-      <c r="G63" s="10"/>
-    </row>
-    <row r="64" spans="7:7">
-      <c r="G64" s="10"/>
-    </row>
-    <row r="65" spans="7:7">
-      <c r="G65" s="10"/>
-    </row>
-    <row r="66" spans="7:7">
-      <c r="G66" s="10"/>
-    </row>
-    <row r="67" spans="7:7">
-      <c r="G67" s="10"/>
-    </row>
-    <row r="68" spans="7:7">
-      <c r="G68" s="10"/>
-    </row>
-    <row r="69" spans="7:7">
-      <c r="G69" s="10"/>
-    </row>
-    <row r="70" spans="7:7">
-      <c r="G70" s="10"/>
-    </row>
-    <row r="71" spans="7:7">
-      <c r="G71" s="10"/>
-    </row>
-    <row r="72" spans="7:7">
-      <c r="G72" s="10"/>
-    </row>
-    <row r="73" spans="7:7">
-      <c r="G73" s="10"/>
-    </row>
-    <row r="74" spans="7:7">
-      <c r="G74" s="10"/>
-    </row>
-    <row r="75" spans="7:7">
-      <c r="G75" s="10"/>
-    </row>
-    <row r="76" spans="7:7">
-      <c r="G76" s="10"/>
-    </row>
-    <row r="77" spans="7:7">
-      <c r="G77" s="10"/>
-    </row>
-    <row r="78" spans="7:7">
-      <c r="G78" s="10"/>
-    </row>
-    <row r="79" spans="7:7">
-      <c r="G79" s="10"/>
-    </row>
-    <row r="80" spans="7:7">
-      <c r="G80" s="10"/>
-    </row>
-    <row r="81" spans="7:7">
-      <c r="G81" s="10"/>
-    </row>
-    <row r="82" spans="7:7">
-      <c r="G82" s="10"/>
-    </row>
-    <row r="83" spans="7:7">
-      <c r="G83" s="10"/>
-    </row>
-    <row r="84" spans="7:7">
-      <c r="G84" s="10"/>
-    </row>
-    <row r="85" spans="7:7">
-      <c r="G85" s="10"/>
-    </row>
-    <row r="86" spans="7:7">
-      <c r="G86" s="10"/>
-    </row>
-    <row r="87" spans="7:7">
-      <c r="G87" s="10"/>
-    </row>
-    <row r="88" spans="7:7">
-      <c r="G88" s="10"/>
-    </row>
-    <row r="89" spans="7:7">
-      <c r="G89" s="10"/>
-    </row>
-    <row r="90" spans="7:7">
-      <c r="G90" s="10"/>
-    </row>
-    <row r="91" spans="7:7">
-      <c r="G91" s="10"/>
-    </row>
-    <row r="92" spans="7:7">
-      <c r="G92" s="10"/>
-    </row>
-    <row r="93" spans="7:7">
-      <c r="G93" s="10"/>
-    </row>
-    <row r="94" spans="7:7">
-      <c r="G94" s="10"/>
-    </row>
-    <row r="95" spans="7:7">
-      <c r="G95" s="10"/>
-    </row>
-    <row r="96" spans="7:7">
-      <c r="G96" s="10"/>
-    </row>
-    <row r="97" spans="7:7">
-      <c r="G97" s="10"/>
-    </row>
-    <row r="98" spans="7:7">
-      <c r="G98" s="10"/>
-    </row>
-    <row r="99" spans="7:7">
-      <c r="G99" s="10"/>
-    </row>
-    <row r="100" spans="7:7">
-      <c r="G100" s="10"/>
+    <row r="32" spans="1:9">
+      <c r="H32" s="10"/>
+    </row>
+    <row r="33" spans="8:8">
+      <c r="H33" s="10"/>
+    </row>
+    <row r="34" spans="8:8">
+      <c r="H34" s="10"/>
+    </row>
+    <row r="35" spans="8:8">
+      <c r="H35" s="10"/>
+    </row>
+    <row r="36" spans="8:8">
+      <c r="H36" s="10"/>
+    </row>
+    <row r="37" spans="8:8">
+      <c r="H37" s="10"/>
+    </row>
+    <row r="38" spans="8:8">
+      <c r="H38" s="10"/>
+    </row>
+    <row r="39" spans="8:8">
+      <c r="H39" s="10"/>
+    </row>
+    <row r="40" spans="8:8">
+      <c r="H40" s="10"/>
+    </row>
+    <row r="41" spans="8:8">
+      <c r="H41" s="10"/>
+    </row>
+    <row r="42" spans="8:8">
+      <c r="H42" s="10"/>
+    </row>
+    <row r="43" spans="8:8">
+      <c r="H43" s="10"/>
+    </row>
+    <row r="44" spans="8:8">
+      <c r="H44" s="10"/>
+    </row>
+    <row r="45" spans="8:8">
+      <c r="H45" s="10"/>
+    </row>
+    <row r="46" spans="8:8">
+      <c r="H46" s="10"/>
+    </row>
+    <row r="47" spans="8:8">
+      <c r="H47" s="10"/>
+    </row>
+    <row r="48" spans="8:8">
+      <c r="H48" s="10"/>
+    </row>
+    <row r="49" spans="8:8">
+      <c r="H49" s="10"/>
+    </row>
+    <row r="50" spans="8:8">
+      <c r="H50" s="10"/>
+    </row>
+    <row r="51" spans="8:8">
+      <c r="H51" s="10"/>
+    </row>
+    <row r="52" spans="8:8">
+      <c r="H52" s="10"/>
+    </row>
+    <row r="53" spans="8:8">
+      <c r="H53" s="10"/>
+    </row>
+    <row r="54" spans="8:8">
+      <c r="H54" s="10"/>
+    </row>
+    <row r="55" spans="8:8">
+      <c r="H55" s="10"/>
+    </row>
+    <row r="56" spans="8:8">
+      <c r="H56" s="10"/>
+    </row>
+    <row r="57" spans="8:8">
+      <c r="H57" s="10"/>
+    </row>
+    <row r="58" spans="8:8">
+      <c r="H58" s="10"/>
+    </row>
+    <row r="59" spans="8:8">
+      <c r="H59" s="10"/>
+    </row>
+    <row r="60" spans="8:8">
+      <c r="H60" s="10"/>
+    </row>
+    <row r="61" spans="8:8">
+      <c r="H61" s="10"/>
+    </row>
+    <row r="62" spans="8:8">
+      <c r="H62" s="10"/>
+    </row>
+    <row r="63" spans="8:8">
+      <c r="H63" s="10"/>
+    </row>
+    <row r="64" spans="8:8">
+      <c r="H64" s="10"/>
+    </row>
+    <row r="65" spans="8:8">
+      <c r="H65" s="10"/>
+    </row>
+    <row r="66" spans="8:8">
+      <c r="H66" s="10"/>
+    </row>
+    <row r="67" spans="8:8">
+      <c r="H67" s="10"/>
+    </row>
+    <row r="68" spans="8:8">
+      <c r="H68" s="10"/>
+    </row>
+    <row r="69" spans="8:8">
+      <c r="H69" s="10"/>
+    </row>
+    <row r="70" spans="8:8">
+      <c r="H70" s="10"/>
+    </row>
+    <row r="71" spans="8:8">
+      <c r="H71" s="10"/>
+    </row>
+    <row r="72" spans="8:8">
+      <c r="H72" s="10"/>
+    </row>
+    <row r="73" spans="8:8">
+      <c r="H73" s="10"/>
+    </row>
+    <row r="74" spans="8:8">
+      <c r="H74" s="10"/>
+    </row>
+    <row r="75" spans="8:8">
+      <c r="H75" s="10"/>
+    </row>
+    <row r="76" spans="8:8">
+      <c r="H76" s="10"/>
+    </row>
+    <row r="77" spans="8:8">
+      <c r="H77" s="10"/>
+    </row>
+    <row r="78" spans="8:8">
+      <c r="H78" s="10"/>
+    </row>
+    <row r="79" spans="8:8">
+      <c r="H79" s="10"/>
+    </row>
+    <row r="80" spans="8:8">
+      <c r="H80" s="10"/>
+    </row>
+    <row r="81" spans="8:8">
+      <c r="H81" s="10"/>
+    </row>
+    <row r="82" spans="8:8">
+      <c r="H82" s="10"/>
+    </row>
+    <row r="83" spans="8:8">
+      <c r="H83" s="10"/>
+    </row>
+    <row r="84" spans="8:8">
+      <c r="H84" s="10"/>
+    </row>
+    <row r="85" spans="8:8">
+      <c r="H85" s="10"/>
+    </row>
+    <row r="86" spans="8:8">
+      <c r="H86" s="10"/>
+    </row>
+    <row r="87" spans="8:8">
+      <c r="H87" s="10"/>
+    </row>
+    <row r="88" spans="8:8">
+      <c r="H88" s="10"/>
+    </row>
+    <row r="89" spans="8:8">
+      <c r="H89" s="10"/>
+    </row>
+    <row r="90" spans="8:8">
+      <c r="H90" s="10"/>
+    </row>
+    <row r="91" spans="8:8">
+      <c r="H91" s="10"/>
+    </row>
+    <row r="92" spans="8:8">
+      <c r="H92" s="10"/>
+    </row>
+    <row r="93" spans="8:8">
+      <c r="H93" s="10"/>
+    </row>
+    <row r="94" spans="8:8">
+      <c r="H94" s="10"/>
+    </row>
+    <row r="95" spans="8:8">
+      <c r="H95" s="10"/>
+    </row>
+    <row r="96" spans="8:8">
+      <c r="H96" s="10"/>
+    </row>
+    <row r="97" spans="8:8">
+      <c r="H97" s="10"/>
+    </row>
+    <row r="98" spans="8:8">
+      <c r="H98" s="10"/>
+    </row>
+    <row r="99" spans="8:8">
+      <c r="H99" s="10"/>
+    </row>
+    <row r="100" spans="8:8">
+      <c r="H100" s="10"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="E2:E200">
+  <conditionalFormatting sqref="F2:F200">
     <cfRule type="expression" dxfId="8" priority="1">
-      <formula>E2="Accepted"</formula>
+      <formula>F2="Accepted"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="7" priority="2">
-      <formula>E2="Pending Review"</formula>
+      <formula>F2="Pending Review"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="6" priority="3">
-      <formula>E2="Rejected"</formula>
+      <formula>F2="Rejected"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="5" priority="4">
-      <formula>E2="Missing"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F200">
-    <cfRule type="expression" dxfId="4" priority="5">
-      <formula>F2="Compliant"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="3" priority="6">
-      <formula>F2="Partially compliant"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="2" priority="7">
-      <formula>F2="Non-compliant"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="1" priority="8">
-      <formula>F2="Not assessed"</formula>
+      <formula>F2="Missing"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G200">
+    <cfRule type="expression" dxfId="4" priority="5">
+      <formula>G2="Compliant"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="3" priority="6">
+      <formula>G2="Partially compliant"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="7">
+      <formula>G2="Non-compliant"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="8">
+      <formula>G2="Not assessed"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H2:H200">
     <cfRule type="expression" dxfId="0" priority="9">
-      <formula>AND(G2&lt;TODAY(),G2&lt;&gt;"")</formula>
+      <formula>AND(H2&lt;TODAY(),H2&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2205,25 +2362,25 @@
           <x14:formula1>
             <xm:f>Reference!$A$2:$A$6</xm:f>
           </x14:formula1>
-          <xm:sqref>B2:B200</xm:sqref>
+          <xm:sqref>C2:C200</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0000-000001000000}">
           <x14:formula1>
             <xm:f>Reference!$D$2:$D$9</xm:f>
           </x14:formula1>
-          <xm:sqref>D2:D200</xm:sqref>
+          <xm:sqref>E2:E200</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0000-000002000000}">
           <x14:formula1>
             <xm:f>Reference!$B$2:$B$5</xm:f>
           </x14:formula1>
-          <xm:sqref>E2:E200</xm:sqref>
+          <xm:sqref>F2:F200</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0000-000003000000}">
           <x14:formula1>
             <xm:f>Reference!$C$2:$C$5</xm:f>
           </x14:formula1>
-          <xm:sqref>F2:F200</xm:sqref>
+          <xm:sqref>G2:G200</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2377,14 +2534,14 @@
         <v>120</v>
       </c>
       <c r="B4" s="14">
-        <f>COUNTA(Evidence_Data!A2:A200)</f>
+        <f>COUNTA(Evidence_Data!B2:B200)</f>
         <v>30</v>
       </c>
       <c r="D4" s="13" t="s">
         <v>13</v>
       </c>
       <c r="E4" s="14">
-        <f>COUNTIF(Evidence_Data!F2:F200,D4)</f>
+        <f>COUNTIF(Evidence_Data!G2:G200,D4)</f>
         <v>13</v>
       </c>
     </row>
@@ -2393,14 +2550,14 @@
         <v>12</v>
       </c>
       <c r="B5" s="14">
-        <f>COUNTIF(Evidence_Data!E2:E200,"Accepted")</f>
+        <f>COUNTIF(Evidence_Data!F2:F200,"Accepted")</f>
         <v>20</v>
       </c>
       <c r="D5" s="13" t="s">
         <v>20</v>
       </c>
       <c r="E5" s="14">
-        <f>COUNTIF(Evidence_Data!F3:F201,D5)</f>
+        <f>COUNTIF(Evidence_Data!G3:G201,D5)</f>
         <v>7</v>
       </c>
     </row>
@@ -2409,14 +2566,14 @@
         <v>25</v>
       </c>
       <c r="B6" s="14">
-        <f>COUNTIF(Evidence_Data!E2:E200,"Pending Review")</f>
+        <f>COUNTIF(Evidence_Data!F2:F200,"Pending Review")</f>
         <v>6</v>
       </c>
       <c r="D6" s="13" t="s">
         <v>35</v>
       </c>
       <c r="E6" s="14">
-        <f>COUNTIF(Evidence_Data!F4:F202,D6)</f>
+        <f>COUNTIF(Evidence_Data!G4:G202,D6)</f>
         <v>5</v>
       </c>
     </row>
@@ -2425,14 +2582,14 @@
         <v>13</v>
       </c>
       <c r="B7" s="14">
-        <f>COUNTIF(Evidence_Data!F2:F200,"Compliant")</f>
+        <f>COUNTIF(Evidence_Data!G2:G200,"Compliant")</f>
         <v>13</v>
       </c>
       <c r="D7" s="15" t="s">
         <v>26</v>
       </c>
       <c r="E7" s="16">
-        <f>COUNTIF(Evidence_Data!F5:F203,D7)</f>
+        <f>COUNTIF(Evidence_Data!G5:G203,D7)</f>
         <v>5</v>
       </c>
     </row>
@@ -2441,7 +2598,7 @@
         <v>20</v>
       </c>
       <c r="B8" s="16">
-        <f>COUNTIF(Evidence_Data!F2:F200,"Partially compliant")</f>
+        <f>COUNTIF(Evidence_Data!G2:G200,"Partially compliant")</f>
         <v>7</v>
       </c>
     </row>
@@ -2456,7 +2613,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="2" width="23" customWidth="1"/>
@@ -2479,114 +2636,136 @@
       </c>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>126</v>
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Document ID</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>documentId</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Document ID</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Stable identifier for the evidence document/row.</t>
+        </is>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="3" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B7" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C7" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D7" s="3" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="28">
-      <c r="A7" s="3" t="s">
+    <row r="8" spans="1:4" ht="28">
+      <c r="A8" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B8" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C8" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D8" s="3" t="s">
         <v>136</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4">
-      <c r="A8" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B10" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C10" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D10" s="3" t="s">
         <v>141</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat:add logic for conflicted clause code
</commit_message>
<xml_diff>
--- a/backend/data/audit_dashboard_excel_simulation_revised.xlsx
+++ b/backend/data/audit_dashboard_excel_simulation_revised.xlsx
@@ -1,21 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nevan\OneDrive\Documents\GitHub\audit-management-dashboard\backend\data\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7531C58-9863-448E-8337-F1DD8E0C774F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500"/>
   </bookViews>
   <sheets>
-    <sheet name="Evidence_Data" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Evidence_Data" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
@@ -55,11 +49,11 @@
     <t>Firewall Configuration Review</t>
   </si>
   <si>
-    <t>ISMS
+    <t xml:space="preserve">ISMS
 PIMS</t>
   </si>
   <si>
-    <t>8.1
+    <t xml:space="preserve">8.1
 8.1</t>
   </si>
   <si>
@@ -99,7 +93,7 @@
     <t>ISMS</t>
   </si>
   <si>
-    <t>8.1, 8.8</t>
+    <t>8.1, A.8.8</t>
   </si>
   <si>
     <t>Singapore</t>
@@ -117,7 +111,7 @@
     <t>Access Control Review</t>
   </si>
   <si>
-    <t>5.15
+    <t xml:space="preserve">A.5.15
 5.15</t>
   </si>
   <si>
@@ -151,11 +145,11 @@
     <t>Business Continuity Test Result</t>
   </si>
   <si>
-    <t>BCMS
+    <t xml:space="preserve">BCMS
 OHSMS</t>
   </si>
   <si>
-    <t>8.5
+    <t xml:space="preserve">8.5
 8.2</t>
   </si>
   <si>
@@ -174,11 +168,11 @@
     <t>Supplier Evaluation Report</t>
   </si>
   <si>
-    <t>EnMS
+    <t xml:space="preserve">EnMS
 ABMS</t>
   </si>
   <si>
-    <t>8.4
+    <t xml:space="preserve">8.4
 8.2</t>
   </si>
   <si>
@@ -194,11 +188,11 @@
     <t>Internal Audit Report Q2</t>
   </si>
   <si>
-    <t>EnMS
+    <t xml:space="preserve">EnMS
 ISMS</t>
   </si>
   <si>
-    <t>9.2
+    <t xml:space="preserve">9.2
 9.2</t>
   </si>
   <si>
@@ -211,7 +205,7 @@
     <t>Risk Treatment Plan</t>
   </si>
   <si>
-    <t>6.1
+    <t xml:space="preserve">6.1
 6.1</t>
   </si>
   <si>
@@ -242,12 +236,12 @@
     <t>Information Security Policy</t>
   </si>
   <si>
-    <t>ISMS
+    <t xml:space="preserve">ISMS
 PIMS
 EnMS</t>
   </si>
   <si>
-    <t>5.2
+    <t xml:space="preserve">5.2
 5.2
 5.2</t>
   </si>
@@ -261,7 +255,7 @@
     <t>Corrective Action Log</t>
   </si>
   <si>
-    <t>10.2
+    <t xml:space="preserve">10.2
 10.2</t>
   </si>
   <si>
@@ -277,11 +271,11 @@
     <t>Disaster Recovery Procedure</t>
   </si>
   <si>
-    <t>BCMS
+    <t xml:space="preserve">BCMS
 ITSMS</t>
   </si>
   <si>
-    <t>8.4
+    <t xml:space="preserve">8.4
 8.4</t>
   </si>
   <si>
@@ -294,12 +288,12 @@
     <t>Security and Compliance Training Record</t>
   </si>
   <si>
-    <t>ISMS
+    <t xml:space="preserve">ISMS
 PIMS
 ABMS</t>
   </si>
   <si>
-    <t>7.2, 7.3
+    <t xml:space="preserve">7.2, 7.3
 7.2
 7.3</t>
   </si>
@@ -313,7 +307,7 @@
     <t>Asset Inventory</t>
   </si>
   <si>
-    <t>5.9</t>
+    <t>A.5.9</t>
   </si>
   <si>
     <t>Japan</t>
@@ -340,11 +334,11 @@
     <t>Management Review Minutes</t>
   </si>
   <si>
-    <t>EnMS
+    <t xml:space="preserve">EnMS
 OHSMS</t>
   </si>
   <si>
-    <t>9.3
+    <t xml:space="preserve">9.3
 9.3</t>
   </si>
   <si>
@@ -384,7 +378,7 @@
     <t>Security Awareness Attendance</t>
   </si>
   <si>
-    <t>6.3
+    <t xml:space="preserve">6.3
 6.3</t>
   </si>
   <si>
@@ -442,7 +436,7 @@
     <t>Penetration Test Report</t>
   </si>
   <si>
-    <t>8.8</t>
+    <t>A.8.8</t>
   </si>
   <si>
     <t>https://contoso.sharepoint.com/sites/AuditEvidence/Documents/penetration-test-report.pdf</t>
@@ -478,7 +472,7 @@
     <t>Business Impact Analysis</t>
   </si>
   <si>
-    <t>8.2
+    <t xml:space="preserve">8.2
 8.2</t>
   </si>
   <si>
@@ -509,19 +503,26 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <color theme="1"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF264C77"/>
       <sz val="11"/>
       <name val="Carlito"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color rgb="FF264C77"/>
       <name val="Carlito"/>
     </font>
   </fonts>
@@ -538,14 +539,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -555,23 +549,20 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+  <cellXfs count="5">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
@@ -582,55 +573,22 @@
     <dxf>
       <font>
         <b/>
-        <color rgb="FFC25A00"/>
+        <color rgb="FF007A55"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFFFF7E0"/>
+          <bgColor rgb="FFE6F8F2"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
         <b/>
-        <color rgb="FF475569"/>
+        <color rgb="FF9A6700"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFF1F5F9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FFB42318"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFDECEC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FFC25A00"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFF7E0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF027A48"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFECFDF3"/>
+          <bgColor rgb="FFFFF4D6"/>
         </patternFill>
       </fill>
     </dxf>
@@ -659,22 +617,55 @@
     <dxf>
       <font>
         <b/>
-        <color rgb="FF9A6700"/>
+        <color rgb="FF027A48"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFFFF4D6"/>
+          <bgColor rgb="FFECFDF3"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
         <b/>
-        <color rgb="FF007A55"/>
+        <color rgb="FFC25A00"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFE6F8F2"/>
+          <bgColor rgb="FFFFF7E0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFB42318"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFDECEC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF475569"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF1F5F9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFC25A00"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFF7E0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -692,17 +683,28 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="EvidenceDashboardTable" displayName="EvidenceDashboardTable" ref="A1:I31">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" name="EvidenceDashboardTable" displayName="EvidenceDashboardTable" ref="A1:I31" totalsRowShown="1" headerRowCount="0">
+  <autoFilter>
+    <filterColumn colId="0" hiddenButton="1"/>
+    <filterColumn colId="1" hiddenButton="1"/>
+    <filterColumn colId="2" hiddenButton="1"/>
+    <filterColumn colId="3" hiddenButton="1"/>
+    <filterColumn colId="4" hiddenButton="1"/>
+    <filterColumn colId="5" hiddenButton="1"/>
+    <filterColumn colId="6" hiddenButton="1"/>
+    <filterColumn colId="7" hiddenButton="1"/>
+    <filterColumn colId="8" hiddenButton="1"/>
+  </autoFilter>
   <tableColumns count="9">
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Evidence ID"/>
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Document/Evidence"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Standard"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Clause"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Location"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Evidence Status"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Compliance Result"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Due Date"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Document URL"/>
+    <tableColumn id="1" name="Evidence ID"/>
+    <tableColumn id="2" name="Document/Evidence"/>
+    <tableColumn id="3" name="Standard"/>
+    <tableColumn id="4" name="Clause"/>
+    <tableColumn id="5" name="Location"/>
+    <tableColumn id="6" name="Evidence Status"/>
+    <tableColumn id="7" name="Compliance Result"/>
+    <tableColumn id="8" name="Due Date"/>
+    <tableColumn id="9" name="Document URL"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -856,9 +858,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I31"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <sheetFormatPr defaultRowHeight="14" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="38" customWidth="1"/>
@@ -869,7 +871,7 @@
     <col min="9" max="9" width="79.58203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="21.4" customHeight="1">
+    <row r="1" ht="21.4" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -891,14 +893,14 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="32" customHeight="1">
+    <row r="2" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
@@ -920,14 +922,14 @@
       <c r="G2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H2" s="5">
+      <c r="H2" s="4">
         <v>46402</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="18" customHeight="1">
+    <row r="3" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>17</v>
       </c>
@@ -949,14 +951,14 @@
       <c r="G3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H3" s="5">
+      <c r="H3" s="4">
         <v>46428</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="18" customHeight="1">
+    <row r="4" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>22</v>
       </c>
@@ -978,14 +980,14 @@
       <c r="G4" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="H4" s="5">
+      <c r="H4" s="4">
         <v>46331</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="32" customHeight="1">
+    <row r="5" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>29</v>
       </c>
@@ -1007,14 +1009,14 @@
       <c r="G5" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="H5" s="5">
+      <c r="H5" s="4">
         <v>46259</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="18" customHeight="1">
+    <row r="6" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>36</v>
       </c>
@@ -1036,14 +1038,14 @@
       <c r="G6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H6" s="5">
+      <c r="H6" s="4">
         <v>46376</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="32" customHeight="1">
+    <row r="7" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>40</v>
       </c>
@@ -1065,14 +1067,14 @@
       <c r="G7" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="H7" s="5">
+      <c r="H7" s="4">
         <v>46204</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="32" customHeight="1">
+    <row r="8" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>47</v>
       </c>
@@ -1094,14 +1096,14 @@
       <c r="G8" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="H8" s="5">
+      <c r="H8" s="4">
         <v>46399</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="32" customHeight="1">
+    <row r="9" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>53</v>
       </c>
@@ -1123,14 +1125,14 @@
       <c r="G9" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="H9" s="5">
+      <c r="H9" s="4">
         <v>46323</v>
       </c>
       <c r="I9" s="2" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="32" customHeight="1">
+    <row r="10" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>58</v>
       </c>
@@ -1152,14 +1154,14 @@
       <c r="G10" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="H10" s="5">
+      <c r="H10" s="4">
         <v>46266</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="18" customHeight="1">
+    <row r="11" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>63</v>
       </c>
@@ -1181,14 +1183,14 @@
       <c r="G11" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H11" s="5">
+      <c r="H11" s="4">
         <v>46464</v>
       </c>
       <c r="I11" s="2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="46" customHeight="1">
+    <row r="12" ht="46" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>68</v>
       </c>
@@ -1210,14 +1212,14 @@
       <c r="G12" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H12" s="5">
+      <c r="H12" s="4">
         <v>46395</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="32" customHeight="1">
+    <row r="13" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>73</v>
       </c>
@@ -1239,14 +1241,14 @@
       <c r="G13" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="H13" s="5">
+      <c r="H13" s="4">
         <v>46235</v>
       </c>
       <c r="I13" s="2" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="32" customHeight="1">
+    <row r="14" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>78</v>
       </c>
@@ -1268,14 +1270,14 @@
       <c r="G14" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H14" s="5">
+      <c r="H14" s="4">
         <v>46378</v>
       </c>
       <c r="I14" s="2" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="46" customHeight="1">
+    <row r="15" ht="46" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>83</v>
       </c>
@@ -1297,14 +1299,14 @@
       <c r="G15" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H15" s="5">
+      <c r="H15" s="4">
         <v>46432</v>
       </c>
       <c r="I15" s="2" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="18" customHeight="1">
+    <row r="16" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>88</v>
       </c>
@@ -1326,14 +1328,14 @@
       <c r="G16" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="H16" s="5">
+      <c r="H16" s="4">
         <v>46193</v>
       </c>
       <c r="I16" s="2" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="18" customHeight="1">
+    <row r="17" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>94</v>
       </c>
@@ -1355,14 +1357,14 @@
       <c r="G17" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="H17" s="5">
+      <c r="H17" s="4">
         <v>46331</v>
       </c>
       <c r="I17" s="2" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="32" customHeight="1">
+    <row r="18" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>97</v>
       </c>
@@ -1384,14 +1386,14 @@
       <c r="G18" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="H18" s="5">
+      <c r="H18" s="4">
         <v>46262</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="18" customHeight="1">
+    <row r="19" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>102</v>
       </c>
@@ -1413,14 +1415,14 @@
       <c r="G19" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H19" s="5">
+      <c r="H19" s="4">
         <v>46476</v>
       </c>
       <c r="I19" s="2" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="18" customHeight="1">
+    <row r="20" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>106</v>
       </c>
@@ -1442,14 +1444,14 @@
       <c r="G20" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="H20" s="5">
+      <c r="H20" s="4">
         <v>46341</v>
       </c>
       <c r="I20" s="2" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="32" customHeight="1">
+    <row r="21" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>111</v>
       </c>
@@ -1471,14 +1473,14 @@
       <c r="G21" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H21" s="5">
+      <c r="H21" s="4">
         <v>46438</v>
       </c>
       <c r="I21" s="2" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="18" customHeight="1">
+    <row r="22" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>115</v>
       </c>
@@ -1500,14 +1502,14 @@
       <c r="G22" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="H22" s="5">
+      <c r="H22" s="4">
         <v>46275</v>
       </c>
       <c r="I22" s="2" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="18" customHeight="1">
+    <row r="23" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>119</v>
       </c>
@@ -1529,14 +1531,14 @@
       <c r="G23" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H23" s="5">
+      <c r="H23" s="4">
         <v>46478</v>
       </c>
       <c r="I23" s="2" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="32" customHeight="1">
+    <row r="24" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>124</v>
       </c>
@@ -1558,14 +1560,14 @@
       <c r="G24" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="H24" s="5">
+      <c r="H24" s="4">
         <v>46223</v>
       </c>
       <c r="I24" s="2" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="18" customHeight="1">
+    <row r="25" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>127</v>
       </c>
@@ -1587,14 +1589,14 @@
       <c r="G25" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H25" s="5">
+      <c r="H25" s="4">
         <v>46348</v>
       </c>
       <c r="I25" s="2" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="18" customHeight="1">
+    <row r="26" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>130</v>
       </c>
@@ -1616,14 +1618,14 @@
       <c r="G26" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="H26" s="5">
+      <c r="H26" s="4">
         <v>46458</v>
       </c>
       <c r="I26" s="2" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="18" customHeight="1">
+    <row r="27" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>134</v>
       </c>
@@ -1645,14 +1647,14 @@
       <c r="G27" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="H27" s="5">
+      <c r="H27" s="4">
         <v>46208</v>
       </c>
       <c r="I27" s="2" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="18" customHeight="1">
+    <row r="28" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>138</v>
       </c>
@@ -1674,14 +1676,14 @@
       <c r="G28" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H28" s="5">
+      <c r="H28" s="4">
         <v>46313</v>
       </c>
       <c r="I28" s="2" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="32" customHeight="1">
+    <row r="29" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>142</v>
       </c>
@@ -1703,14 +1705,14 @@
       <c r="G29" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="H29" s="5">
+      <c r="H29" s="4">
         <v>46270</v>
       </c>
       <c r="I29" s="2" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="18" customHeight="1">
+    <row r="30" ht="18" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>146</v>
       </c>
@@ -1732,14 +1734,14 @@
       <c r="G30" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H30" s="5">
+      <c r="H30" s="4">
         <v>46356</v>
       </c>
       <c r="I30" s="2" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="32" customHeight="1">
+    <row r="31" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>150</v>
       </c>
@@ -1761,7 +1763,7 @@
       <c r="G31" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="H31" s="5">
+      <c r="H31" s="4">
         <v>46426</v>
       </c>
       <c r="I31" s="2" t="s">
@@ -1770,16 +1772,16 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F200">
-    <cfRule type="expression" dxfId="8" priority="1">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>F2="Accepted"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="2">
+    <cfRule type="expression" dxfId="1" priority="2">
       <formula>F2="Pending Review"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="3">
+    <cfRule type="expression" dxfId="2" priority="3">
       <formula>F2="Rejected"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="4">
+    <cfRule type="expression" dxfId="3" priority="4">
       <formula>F2="Missing"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1787,18 +1789,18 @@
     <cfRule type="expression" dxfId="4" priority="5">
       <formula>G2="Compliant"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="6">
+    <cfRule type="expression" dxfId="5" priority="6">
       <formula>G2="Partially compliant"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="7">
+    <cfRule type="expression" dxfId="6" priority="7">
       <formula>G2="Non-compliant"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="8">
+    <cfRule type="expression" dxfId="7" priority="8">
       <formula>G2="Not assessed"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H200">
-    <cfRule type="expression" dxfId="0" priority="9">
+    <cfRule type="expression" dxfId="8" priority="9">
       <formula>AND(H2&lt;TODAY(),H2&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>